<commit_message>
Desafio 2 - Desafio 4
</commit_message>
<xml_diff>
--- a/Desafio 4 - Vale Refeição/Desafio 4 - Dados - I2A2/DESLIGADOS sem sindicato.xlsx
+++ b/Desafio 4 - Vale Refeição/Desafio 4 - Dados - I2A2/DESLIGADOS sem sindicato.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Meu Drive\Cursos e Treinamentos\Cientista de Dados\Treinamento Python\I2A2\Desafios\Desafio 4 - Vale Refeição\Desafio 4 - Dados - I2A2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC2CFAE-1DFE-4644-A53C-28E8EF1E7176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA852EAF-8615-4B73-89B3-C8A870FBED27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1475C584-71FD-435B-B4EE-9C19DEBEC6B0}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="5">
   <si>
     <t>DATA DEMISSÃO</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t>MATRICULA</t>
+  </si>
+  <si>
+    <t>Sindicatos</t>
   </si>
 </sst>
 </file>
@@ -461,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C6A81D-95CF-4A37-B9C3-5DE934ECBCD1}">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultColWidth="52.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -469,7 +472,7 @@
     <col min="3" max="3" width="33.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -479,8 +482,11 @@
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>34706</v>
       </c>
@@ -491,7 +497,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>31486</v>
       </c>
@@ -502,7 +508,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>34641</v>
       </c>
@@ -513,7 +519,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>26139</v>
       </c>
@@ -524,7 +530,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>34179</v>
       </c>
@@ -535,7 +541,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>33482</v>
       </c>
@@ -546,7 +552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>33492</v>
       </c>
@@ -555,7 +561,7 @@
       </c>
       <c r="C8" s="5"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>33627</v>
       </c>
@@ -566,7 +572,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>33404</v>
       </c>
@@ -577,7 +583,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>33922</v>
       </c>
@@ -588,7 +594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>25707</v>
       </c>
@@ -599,7 +605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>34935</v>
       </c>
@@ -610,7 +616,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>33989</v>
       </c>
@@ -621,7 +627,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>29294</v>
       </c>
@@ -632,7 +638,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>31394</v>
       </c>

</xml_diff>